<commit_message>
Actualizacion automatica mar 22/09/2026 11:36:41.85
</commit_message>
<xml_diff>
--- a/data/BD Personal.xlsx
+++ b/data/BD Personal.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://apoyoconsultoria0.sharepoint.com/sites/fileserver/Polticas Pblicas/6 Proyectos/2025/2025-070-O IJM - Linea de base/04. Analisis/03. Programacion/06. Dashboard Seguimiento Web/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="21" documentId="11_A10BAE44CD785D61F5141092B1107384533E0B90" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{78D69169-60F1-420D-BB87-B4C6C30E1148}"/>
+  <xr:revisionPtr revIDLastSave="24" documentId="11_A10BAE44CD785D61F5141092B1107384533E0B90" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{40AD01C3-1CB7-49F0-BD5E-DC808AEC213E}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="157">
   <si>
     <t>CODPER</t>
   </si>
@@ -503,10 +503,10 @@
     <t>SAGRARIO MAGNOLIA ORTIZ MOLLEPAZA</t>
   </si>
   <si>
-    <t>C1</t>
-  </si>
-  <si>
     <t>JENNY SALON ANAHUA</t>
+  </si>
+  <si>
+    <t>C0</t>
   </si>
 </sst>
 </file>
@@ -1074,6 +1074,12 @@
       <c r="D14" t="s">
         <v>23</v>
       </c>
+      <c r="E14" t="s">
+        <v>39</v>
+      </c>
+      <c r="F14" s="2">
+        <v>46252</v>
+      </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15">
@@ -2583,10 +2589,10 @@
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
+        <v>156</v>
+      </c>
+      <c r="B120" t="s">
         <v>155</v>
-      </c>
-      <c r="B120" t="s">
-        <v>156</v>
       </c>
       <c r="C120" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
Actualizacion automatica mié 23/09/2026  8:54:25.38
</commit_message>
<xml_diff>
--- a/data/BD Personal.xlsx
+++ b/data/BD Personal.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://apoyoconsultoria0.sharepoint.com/sites/fileserver/Polticas Pblicas/6 Proyectos/2025/2025-070-O IJM - Linea de base/04. Analisis/03. Programacion/06. Dashboard Seguimiento Web/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="24" documentId="11_A10BAE44CD785D61F5141092B1107384533E0B90" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{40AD01C3-1CB7-49F0-BD5E-DC808AEC213E}"/>
+  <xr:revisionPtr revIDLastSave="30" documentId="11_A10BAE44CD785D61F5141092B1107384533E0B90" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{44CD5B62-7048-40D7-B0C9-7AD4ED1706F7}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="5748" yWindow="348" windowWidth="11712" windowHeight="12240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Exported" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Exported!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Exported!$A$1:$F$120</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -863,6 +863,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:F120"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -893,7 +894,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -907,7 +908,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -921,7 +922,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -935,7 +936,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -949,7 +950,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -963,7 +964,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -977,7 +978,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -991,7 +992,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1005,7 +1006,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1019,7 +1020,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1033,7 +1034,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1047,7 +1048,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1061,7 +1062,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1081,7 +1082,7 @@
         <v>46252</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1095,7 +1096,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1109,7 +1110,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1129,7 +1130,7 @@
         <v>46252</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1143,7 +1144,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1157,7 +1158,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1171,7 +1172,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1185,7 +1186,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1199,7 +1200,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1213,7 +1214,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1227,7 +1228,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1241,7 +1242,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1255,7 +1256,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1269,7 +1270,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1289,7 +1290,7 @@
         <v>46253</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1303,7 +1304,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1317,7 +1318,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1331,7 +1332,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1345,7 +1346,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1359,7 +1360,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>33</v>
       </c>
@@ -1373,7 +1374,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>34</v>
       </c>
@@ -1387,7 +1388,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>35</v>
       </c>
@@ -1401,7 +1402,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>36</v>
       </c>
@@ -1415,7 +1416,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>37</v>
       </c>
@@ -1429,7 +1430,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>38</v>
       </c>
@@ -1443,7 +1444,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>39</v>
       </c>
@@ -1457,7 +1458,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>40</v>
       </c>
@@ -1471,7 +1472,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>41</v>
       </c>
@@ -1485,7 +1486,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>42</v>
       </c>
@@ -1499,7 +1500,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>43</v>
       </c>
@@ -1513,7 +1514,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>44</v>
       </c>
@@ -1527,7 +1528,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>45</v>
       </c>
@@ -1541,7 +1542,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>46</v>
       </c>
@@ -1555,7 +1556,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>47</v>
       </c>
@@ -1569,7 +1570,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>48</v>
       </c>
@@ -1583,7 +1584,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>50</v>
       </c>
@@ -1597,7 +1598,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>51</v>
       </c>
@@ -1611,7 +1612,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>52</v>
       </c>
@@ -1625,7 +1626,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>53</v>
       </c>
@@ -1639,7 +1640,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>54</v>
       </c>
@@ -1653,7 +1654,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>55</v>
       </c>
@@ -1667,7 +1668,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>56</v>
       </c>
@@ -1681,7 +1682,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>57</v>
       </c>
@@ -1695,7 +1696,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>58</v>
       </c>
@@ -1709,7 +1710,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>59</v>
       </c>
@@ -1723,7 +1724,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>60</v>
       </c>
@@ -1737,7 +1738,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>61</v>
       </c>
@@ -1751,7 +1752,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>62</v>
       </c>
@@ -1765,7 +1766,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>63</v>
       </c>
@@ -1779,7 +1780,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>64</v>
       </c>
@@ -1793,7 +1794,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>65</v>
       </c>
@@ -1807,7 +1808,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>66</v>
       </c>
@@ -1821,7 +1822,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>67</v>
       </c>
@@ -1835,7 +1836,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>68</v>
       </c>
@@ -1855,7 +1856,7 @@
         <v>46252</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>69</v>
       </c>
@@ -1869,7 +1870,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>70</v>
       </c>
@@ -1889,7 +1890,7 @@
         <v>46251</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>71</v>
       </c>
@@ -1903,7 +1904,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>72</v>
       </c>
@@ -1917,7 +1918,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>73</v>
       </c>
@@ -1931,7 +1932,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>74</v>
       </c>
@@ -1945,7 +1946,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>75</v>
       </c>
@@ -1959,7 +1960,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>76</v>
       </c>
@@ -1973,7 +1974,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>77</v>
       </c>
@@ -1987,7 +1988,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>78</v>
       </c>
@@ -2001,7 +2002,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>79</v>
       </c>
@@ -2015,7 +2016,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>80</v>
       </c>
@@ -2029,7 +2030,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>81</v>
       </c>
@@ -2043,7 +2044,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>82</v>
       </c>
@@ -2057,7 +2058,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A83">
         <v>83</v>
       </c>
@@ -2071,7 +2072,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A84">
         <v>84</v>
       </c>
@@ -2085,7 +2086,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>85</v>
       </c>
@@ -2099,7 +2100,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>86</v>
       </c>
@@ -2113,7 +2114,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>87</v>
       </c>
@@ -2127,7 +2128,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>88</v>
       </c>
@@ -2141,7 +2142,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A89">
         <v>89</v>
       </c>
@@ -2155,7 +2156,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A90">
         <v>90</v>
       </c>
@@ -2169,7 +2170,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A91">
         <v>91</v>
       </c>
@@ -2197,7 +2198,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A93">
         <v>93</v>
       </c>
@@ -2211,7 +2212,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A94">
         <v>94</v>
       </c>
@@ -2225,7 +2226,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A95">
         <v>95</v>
       </c>
@@ -2239,7 +2240,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A96">
         <v>96</v>
       </c>
@@ -2253,7 +2254,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A97">
         <v>97</v>
       </c>
@@ -2267,7 +2268,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A98">
         <v>98</v>
       </c>
@@ -2287,7 +2288,7 @@
         <v>46224</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A99">
         <v>99</v>
       </c>
@@ -2301,7 +2302,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>114</v>
       </c>
@@ -2321,7 +2322,7 @@
         <v>46253</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>117</v>
       </c>
@@ -2335,7 +2336,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>119</v>
       </c>
@@ -2349,7 +2350,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>121</v>
       </c>
@@ -2363,7 +2364,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>123</v>
       </c>
@@ -2377,7 +2378,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>125</v>
       </c>
@@ -2391,7 +2392,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>127</v>
       </c>
@@ -2405,7 +2406,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>129</v>
       </c>
@@ -2419,7 +2420,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>131</v>
       </c>
@@ -2433,7 +2434,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>133</v>
       </c>
@@ -2447,7 +2448,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>135</v>
       </c>
@@ -2461,7 +2462,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>137</v>
       </c>
@@ -2475,7 +2476,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>139</v>
       </c>
@@ -2489,7 +2490,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>141</v>
       </c>
@@ -2503,7 +2504,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>143</v>
       </c>
@@ -2517,7 +2518,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>145</v>
       </c>
@@ -2531,7 +2532,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>147</v>
       </c>
@@ -2545,7 +2546,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>149</v>
       </c>
@@ -2559,7 +2560,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>151</v>
       </c>
@@ -2573,7 +2574,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>153</v>
       </c>
@@ -2587,7 +2588,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>156</v>
       </c>
@@ -2602,20 +2603,18 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:F120" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="Veronica Aulla Acuña"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="667d70cb-f49f-4223-87b6-a8a0e4fc3231">
@@ -2624,6 +2623,15 @@
     <TaxCatchAll xmlns="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2834,20 +2842,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{630299A7-E824-4D69-AA5E-3193E7062408}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E73E3A5A-F8DC-40E4-A1F8-9A051C36DEF4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="667d70cb-f49f-4223-87b6-a8a0e4fc3231"/>
     <ds:schemaRef ds:uri="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{630299A7-E824-4D69-AA5E-3193E7062408}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Actualizacion automatica mié 30/09/2026  8:52:48.47
</commit_message>
<xml_diff>
--- a/data/BD Personal.xlsx
+++ b/data/BD Personal.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://apoyoconsultoria0.sharepoint.com/sites/fileserver/Polticas Pblicas/6 Proyectos/2025/2025-070-O IJM - Linea de base/04. Analisis/03. Programacion/06. Dashboard Seguimiento Web/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="30" documentId="11_A10BAE44CD785D61F5141092B1107384533E0B90" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{44CD5B62-7048-40D7-B0C9-7AD4ED1706F7}"/>
+  <xr:revisionPtr revIDLastSave="33" documentId="11_A10BAE44CD785D61F5141092B1107384533E0B90" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{648D3667-DD17-4869-9AE5-0B7034ED7681}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="5748" yWindow="348" windowWidth="11712" windowHeight="12240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Exported" sheetId="1" r:id="rId1"/>
@@ -863,7 +863,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:F120"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -894,7 +893,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -908,7 +907,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -922,7 +921,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -936,7 +935,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -950,7 +949,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -964,7 +963,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -978,7 +977,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -992,7 +991,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1006,7 +1005,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1020,7 +1019,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1034,7 +1033,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1048,7 +1047,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1062,7 +1061,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1082,7 +1081,7 @@
         <v>46252</v>
       </c>
     </row>
-    <row r="15" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1096,7 +1095,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="16" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1110,7 +1109,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="17" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1130,7 +1129,7 @@
         <v>46252</v>
       </c>
     </row>
-    <row r="18" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1144,7 +1143,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1158,7 +1157,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="20" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1172,7 +1171,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="21" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1186,7 +1185,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="22" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1200,7 +1199,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="23" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1214,7 +1213,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="24" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1228,7 +1227,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="25" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1242,7 +1241,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="26" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1256,7 +1255,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="27" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1270,7 +1269,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="28" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1290,7 +1289,7 @@
         <v>46253</v>
       </c>
     </row>
-    <row r="29" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1304,7 +1303,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="30" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1318,7 +1317,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="31" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1332,7 +1331,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="32" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1346,7 +1345,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="33" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1360,7 +1359,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="34" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>33</v>
       </c>
@@ -1374,7 +1373,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="35" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>34</v>
       </c>
@@ -1388,7 +1387,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="36" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>35</v>
       </c>
@@ -1402,7 +1401,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="37" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>36</v>
       </c>
@@ -1416,7 +1415,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="38" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>37</v>
       </c>
@@ -1430,7 +1429,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="39" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>38</v>
       </c>
@@ -1444,7 +1443,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="40" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>39</v>
       </c>
@@ -1458,7 +1457,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="41" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>40</v>
       </c>
@@ -1472,7 +1471,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="42" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>41</v>
       </c>
@@ -1486,7 +1485,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="43" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>42</v>
       </c>
@@ -1500,7 +1499,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="44" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>43</v>
       </c>
@@ -1514,7 +1513,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="45" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>44</v>
       </c>
@@ -1528,7 +1527,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="46" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>45</v>
       </c>
@@ -1542,7 +1541,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="47" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>46</v>
       </c>
@@ -1556,7 +1555,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="48" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>47</v>
       </c>
@@ -1570,7 +1569,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="49" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>48</v>
       </c>
@@ -1584,7 +1583,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="50" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>50</v>
       </c>
@@ -1598,7 +1597,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="51" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>51</v>
       </c>
@@ -1612,7 +1611,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="52" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>52</v>
       </c>
@@ -1626,7 +1625,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="53" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>53</v>
       </c>
@@ -1640,7 +1639,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="54" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>54</v>
       </c>
@@ -1654,7 +1653,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="55" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>55</v>
       </c>
@@ -1668,7 +1667,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="56" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>56</v>
       </c>
@@ -1682,7 +1681,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="57" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>57</v>
       </c>
@@ -1696,7 +1695,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="58" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>58</v>
       </c>
@@ -1710,7 +1709,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="59" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>59</v>
       </c>
@@ -1724,7 +1723,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="60" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>60</v>
       </c>
@@ -1738,7 +1737,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="61" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>61</v>
       </c>
@@ -1752,7 +1751,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="62" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>62</v>
       </c>
@@ -1766,7 +1765,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="63" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>63</v>
       </c>
@@ -1780,7 +1779,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="64" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>64</v>
       </c>
@@ -1794,7 +1793,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="65" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>65</v>
       </c>
@@ -1808,7 +1807,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="66" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>66</v>
       </c>
@@ -1822,7 +1821,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="67" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>67</v>
       </c>
@@ -1836,7 +1835,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="68" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>68</v>
       </c>
@@ -1856,7 +1855,7 @@
         <v>46252</v>
       </c>
     </row>
-    <row r="69" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>69</v>
       </c>
@@ -1870,7 +1869,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="70" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>70</v>
       </c>
@@ -1890,7 +1889,7 @@
         <v>46251</v>
       </c>
     </row>
-    <row r="71" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>71</v>
       </c>
@@ -1904,7 +1903,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="72" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>72</v>
       </c>
@@ -1918,7 +1917,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="73" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>73</v>
       </c>
@@ -1932,7 +1931,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="74" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>74</v>
       </c>
@@ -1946,7 +1945,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="75" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>75</v>
       </c>
@@ -1960,7 +1959,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="76" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>76</v>
       </c>
@@ -1974,7 +1973,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="77" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>77</v>
       </c>
@@ -1988,7 +1987,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="78" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>78</v>
       </c>
@@ -2002,7 +2001,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="79" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>79</v>
       </c>
@@ -2016,7 +2015,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="80" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>80</v>
       </c>
@@ -2030,7 +2029,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="81" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>81</v>
       </c>
@@ -2044,7 +2043,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="82" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>82</v>
       </c>
@@ -2058,7 +2057,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="83" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A83">
         <v>83</v>
       </c>
@@ -2072,7 +2071,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="84" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A84">
         <v>84</v>
       </c>
@@ -2086,7 +2085,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="85" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>85</v>
       </c>
@@ -2100,7 +2099,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="86" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>86</v>
       </c>
@@ -2114,7 +2113,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="87" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>87</v>
       </c>
@@ -2128,7 +2127,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="88" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>88</v>
       </c>
@@ -2142,7 +2141,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="89" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A89">
         <v>89</v>
       </c>
@@ -2156,7 +2155,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="90" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A90">
         <v>90</v>
       </c>
@@ -2170,7 +2169,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="91" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A91">
         <v>91</v>
       </c>
@@ -2198,7 +2197,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="93" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A93">
         <v>93</v>
       </c>
@@ -2212,7 +2211,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="94" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A94">
         <v>94</v>
       </c>
@@ -2226,7 +2225,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="95" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A95">
         <v>95</v>
       </c>
@@ -2240,7 +2239,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="96" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A96">
         <v>96</v>
       </c>
@@ -2254,7 +2253,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="97" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A97">
         <v>97</v>
       </c>
@@ -2268,7 +2267,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="98" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A98">
         <v>98</v>
       </c>
@@ -2288,7 +2287,7 @@
         <v>46224</v>
       </c>
     </row>
-    <row r="99" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A99">
         <v>99</v>
       </c>
@@ -2302,7 +2301,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="100" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>114</v>
       </c>
@@ -2322,7 +2321,7 @@
         <v>46253</v>
       </c>
     </row>
-    <row r="101" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>117</v>
       </c>
@@ -2336,7 +2335,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="102" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>119</v>
       </c>
@@ -2350,7 +2349,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="103" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>121</v>
       </c>
@@ -2364,7 +2363,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="104" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>123</v>
       </c>
@@ -2378,7 +2377,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="105" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>125</v>
       </c>
@@ -2392,7 +2391,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="106" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>127</v>
       </c>
@@ -2406,7 +2405,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="107" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>129</v>
       </c>
@@ -2420,7 +2419,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="108" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>131</v>
       </c>
@@ -2434,7 +2433,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="109" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>133</v>
       </c>
@@ -2448,7 +2447,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="110" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>135</v>
       </c>
@@ -2462,7 +2461,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="111" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>137</v>
       </c>
@@ -2476,7 +2475,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="112" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>139</v>
       </c>
@@ -2490,7 +2489,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="113" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>141</v>
       </c>
@@ -2504,7 +2503,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="114" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>143</v>
       </c>
@@ -2518,7 +2517,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="115" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>145</v>
       </c>
@@ -2532,7 +2531,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="116" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>147</v>
       </c>
@@ -2546,7 +2545,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="117" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>149</v>
       </c>
@@ -2560,7 +2559,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="118" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>151</v>
       </c>
@@ -2574,7 +2573,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="119" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>153</v>
       </c>
@@ -2588,7 +2587,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="120" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>156</v>
       </c>
@@ -2603,18 +2602,20 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F120" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="1">
-      <filters>
-        <filter val="Veronica Aulla Acuña"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="667d70cb-f49f-4223-87b6-a8a0e4fc3231">
@@ -2623,15 +2624,6 @@
     <TaxCatchAll xmlns="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2842,20 +2834,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{630299A7-E824-4D69-AA5E-3193E7062408}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E73E3A5A-F8DC-40E4-A1F8-9A051C36DEF4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="667d70cb-f49f-4223-87b6-a8a0e4fc3231"/>
     <ds:schemaRef ds:uri="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{630299A7-E824-4D69-AA5E-3193E7062408}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Actualizacion automatica vie 02/10/2026  9:11:46.32
</commit_message>
<xml_diff>
--- a/data/BD Personal.xlsx
+++ b/data/BD Personal.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://apoyoconsultoria0.sharepoint.com/sites/fileserver/Polticas Pblicas/6 Proyectos/2025/2025-070-O IJM - Linea de base/04. Analisis/03. Programacion/06. Dashboard Seguimiento Web/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="33" documentId="11_A10BAE44CD785D61F5141092B1107384533E0B90" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{648D3667-DD17-4869-9AE5-0B7034ED7681}"/>
+  <xr:revisionPtr revIDLastSave="35" documentId="11_A10BAE44CD785D61F5141092B1107384533E0B90" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4DCEF9D0-7FA4-46F3-80B4-095187A9D4B3}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -863,6 +863,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:F120"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -893,7 +894,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -907,7 +908,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -921,7 +922,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -935,7 +936,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -949,7 +950,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -963,7 +964,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -977,7 +978,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -991,7 +992,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1005,7 +1006,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1019,7 +1020,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1033,7 +1034,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1047,7 +1048,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1061,7 +1062,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1081,7 +1082,7 @@
         <v>46252</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1095,7 +1096,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1109,7 +1110,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1129,7 +1130,7 @@
         <v>46252</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1143,7 +1144,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1157,7 +1158,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1171,7 +1172,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1185,7 +1186,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1199,7 +1200,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1213,7 +1214,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1227,7 +1228,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1241,7 +1242,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1255,7 +1256,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1289,7 +1290,7 @@
         <v>46253</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1303,7 +1304,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1317,7 +1318,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1331,7 +1332,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1345,7 +1346,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1359,7 +1360,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>33</v>
       </c>
@@ -1373,7 +1374,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>34</v>
       </c>
@@ -1387,7 +1388,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>35</v>
       </c>
@@ -1401,7 +1402,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>36</v>
       </c>
@@ -1415,7 +1416,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>37</v>
       </c>
@@ -1429,7 +1430,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>38</v>
       </c>
@@ -1443,7 +1444,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>39</v>
       </c>
@@ -1457,7 +1458,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>40</v>
       </c>
@@ -1471,7 +1472,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>41</v>
       </c>
@@ -1485,7 +1486,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>42</v>
       </c>
@@ -1499,7 +1500,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>43</v>
       </c>
@@ -1513,7 +1514,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>44</v>
       </c>
@@ -1527,7 +1528,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>45</v>
       </c>
@@ -1541,7 +1542,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>46</v>
       </c>
@@ -1555,7 +1556,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>47</v>
       </c>
@@ -1569,7 +1570,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>48</v>
       </c>
@@ -1583,7 +1584,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>50</v>
       </c>
@@ -1597,7 +1598,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>51</v>
       </c>
@@ -1611,7 +1612,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>52</v>
       </c>
@@ -1625,7 +1626,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>53</v>
       </c>
@@ -1639,7 +1640,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>54</v>
       </c>
@@ -1653,7 +1654,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>55</v>
       </c>
@@ -1667,7 +1668,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>56</v>
       </c>
@@ -1681,7 +1682,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>57</v>
       </c>
@@ -1695,7 +1696,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>58</v>
       </c>
@@ -1709,7 +1710,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>59</v>
       </c>
@@ -1723,7 +1724,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>60</v>
       </c>
@@ -1737,7 +1738,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>61</v>
       </c>
@@ -1751,7 +1752,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>62</v>
       </c>
@@ -1765,7 +1766,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>63</v>
       </c>
@@ -1779,7 +1780,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>64</v>
       </c>
@@ -1793,7 +1794,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>65</v>
       </c>
@@ -1807,7 +1808,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>66</v>
       </c>
@@ -1821,7 +1822,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>67</v>
       </c>
@@ -1835,7 +1836,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>68</v>
       </c>
@@ -1855,7 +1856,7 @@
         <v>46252</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>69</v>
       </c>
@@ -1869,7 +1870,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>70</v>
       </c>
@@ -1889,7 +1890,7 @@
         <v>46251</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>71</v>
       </c>
@@ -1903,7 +1904,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>72</v>
       </c>
@@ -1917,7 +1918,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>73</v>
       </c>
@@ -1931,7 +1932,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>74</v>
       </c>
@@ -1945,7 +1946,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>75</v>
       </c>
@@ -1959,7 +1960,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>76</v>
       </c>
@@ -1973,7 +1974,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>77</v>
       </c>
@@ -1987,7 +1988,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>78</v>
       </c>
@@ -2001,7 +2002,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>79</v>
       </c>
@@ -2015,7 +2016,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>80</v>
       </c>
@@ -2029,7 +2030,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>81</v>
       </c>
@@ -2043,7 +2044,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>82</v>
       </c>
@@ -2057,7 +2058,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A83">
         <v>83</v>
       </c>
@@ -2071,7 +2072,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A84">
         <v>84</v>
       </c>
@@ -2085,7 +2086,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>85</v>
       </c>
@@ -2099,7 +2100,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>86</v>
       </c>
@@ -2113,7 +2114,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>87</v>
       </c>
@@ -2127,7 +2128,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>88</v>
       </c>
@@ -2141,7 +2142,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A89">
         <v>89</v>
       </c>
@@ -2155,7 +2156,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A90">
         <v>90</v>
       </c>
@@ -2169,7 +2170,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A91">
         <v>91</v>
       </c>
@@ -2183,7 +2184,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A92">
         <v>92</v>
       </c>
@@ -2197,7 +2198,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A93">
         <v>93</v>
       </c>
@@ -2211,7 +2212,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A94">
         <v>94</v>
       </c>
@@ -2225,7 +2226,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A95">
         <v>95</v>
       </c>
@@ -2239,7 +2240,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A96">
         <v>96</v>
       </c>
@@ -2253,7 +2254,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A97">
         <v>97</v>
       </c>
@@ -2267,7 +2268,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A98">
         <v>98</v>
       </c>
@@ -2287,7 +2288,7 @@
         <v>46224</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A99">
         <v>99</v>
       </c>
@@ -2301,7 +2302,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>114</v>
       </c>
@@ -2321,7 +2322,7 @@
         <v>46253</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>117</v>
       </c>
@@ -2335,7 +2336,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>119</v>
       </c>
@@ -2349,7 +2350,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>121</v>
       </c>
@@ -2363,7 +2364,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>123</v>
       </c>
@@ -2377,7 +2378,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>125</v>
       </c>
@@ -2391,7 +2392,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>127</v>
       </c>
@@ -2405,7 +2406,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>129</v>
       </c>
@@ -2419,7 +2420,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>131</v>
       </c>
@@ -2433,7 +2434,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>133</v>
       </c>
@@ -2447,7 +2448,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>135</v>
       </c>
@@ -2461,7 +2462,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>137</v>
       </c>
@@ -2475,7 +2476,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>139</v>
       </c>
@@ -2489,7 +2490,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>141</v>
       </c>
@@ -2503,7 +2504,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>143</v>
       </c>
@@ -2517,7 +2518,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>145</v>
       </c>
@@ -2531,7 +2532,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>147</v>
       </c>
@@ -2545,7 +2546,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>149</v>
       </c>
@@ -2559,7 +2560,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>151</v>
       </c>
@@ -2573,7 +2574,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>153</v>
       </c>
@@ -2587,7 +2588,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>156</v>
       </c>
@@ -2602,20 +2603,18 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:F120" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="Jovita Alvarado Rafael"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="667d70cb-f49f-4223-87b6-a8a0e4fc3231">
@@ -2624,6 +2623,15 @@
     <TaxCatchAll xmlns="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2834,20 +2842,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{630299A7-E824-4D69-AA5E-3193E7062408}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E73E3A5A-F8DC-40E4-A1F8-9A051C36DEF4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="667d70cb-f49f-4223-87b6-a8a0e4fc3231"/>
     <ds:schemaRef ds:uri="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{630299A7-E824-4D69-AA5E-3193E7062408}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Actualizacion automatica vie 09/10/2026  9:58:02.09
</commit_message>
<xml_diff>
--- a/data/BD Personal.xlsx
+++ b/data/BD Personal.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://apoyoconsultoria0.sharepoint.com/sites/fileserver/Polticas Pblicas/6 Proyectos/2025/2025-070-O IJM - Linea de base/04. Analisis/03. Programacion/06. Dashboard Seguimiento Web/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="35" documentId="11_A10BAE44CD785D61F5141092B1107384533E0B90" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4DCEF9D0-7FA4-46F3-80B4-095187A9D4B3}"/>
+  <xr:revisionPtr revIDLastSave="41" documentId="11_A10BAE44CD785D61F5141092B1107384533E0B90" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F9295F5B-D81C-4CB2-888E-5597E2499581}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="157">
   <si>
     <t>CODPER</t>
   </si>
@@ -863,7 +863,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:F120"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -894,7 +893,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -908,7 +907,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -922,7 +921,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -936,7 +935,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -950,7 +949,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -964,7 +963,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -978,7 +977,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -992,7 +991,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1006,7 +1005,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1020,7 +1019,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1034,7 +1033,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1048,7 +1047,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1062,7 +1061,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1082,7 +1081,7 @@
         <v>46252</v>
       </c>
     </row>
-    <row r="15" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1096,7 +1095,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="16" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1110,7 +1109,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="17" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1130,7 +1129,7 @@
         <v>46252</v>
       </c>
     </row>
-    <row r="18" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1144,7 +1143,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1158,7 +1157,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="20" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1172,7 +1171,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="21" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1186,7 +1185,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="22" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1200,7 +1199,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="23" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1214,7 +1213,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="24" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1228,7 +1227,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="25" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1242,7 +1241,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="26" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1256,7 +1255,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="27" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1290,7 +1289,7 @@
         <v>46253</v>
       </c>
     </row>
-    <row r="29" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1304,7 +1303,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="30" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1318,7 +1317,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="31" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1332,7 +1331,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="32" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1346,7 +1345,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="33" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1360,7 +1359,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="34" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>33</v>
       </c>
@@ -1374,7 +1373,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="35" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>34</v>
       </c>
@@ -1388,7 +1387,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="36" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>35</v>
       </c>
@@ -1402,7 +1401,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="37" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>36</v>
       </c>
@@ -1416,7 +1415,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="38" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>37</v>
       </c>
@@ -1430,7 +1429,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="39" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>38</v>
       </c>
@@ -1444,7 +1443,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="40" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>39</v>
       </c>
@@ -1458,7 +1457,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="41" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>40</v>
       </c>
@@ -1472,7 +1471,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="42" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>41</v>
       </c>
@@ -1486,7 +1485,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="43" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>42</v>
       </c>
@@ -1500,7 +1499,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="44" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>43</v>
       </c>
@@ -1514,7 +1513,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="45" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>44</v>
       </c>
@@ -1528,7 +1527,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="46" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>45</v>
       </c>
@@ -1542,7 +1541,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="47" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>46</v>
       </c>
@@ -1556,7 +1555,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="48" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>47</v>
       </c>
@@ -1570,7 +1569,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="49" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>48</v>
       </c>
@@ -1584,7 +1583,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="50" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>50</v>
       </c>
@@ -1598,7 +1597,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="51" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>51</v>
       </c>
@@ -1612,7 +1611,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="52" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>52</v>
       </c>
@@ -1626,7 +1625,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="53" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>53</v>
       </c>
@@ -1640,7 +1639,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="54" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>54</v>
       </c>
@@ -1654,7 +1653,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="55" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>55</v>
       </c>
@@ -1668,7 +1667,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="56" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>56</v>
       </c>
@@ -1682,7 +1681,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="57" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>57</v>
       </c>
@@ -1696,7 +1695,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="58" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>58</v>
       </c>
@@ -1710,7 +1709,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="59" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>59</v>
       </c>
@@ -1724,7 +1723,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="60" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>60</v>
       </c>
@@ -1738,7 +1737,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="61" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>61</v>
       </c>
@@ -1752,7 +1751,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="62" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>62</v>
       </c>
@@ -1766,7 +1765,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="63" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>63</v>
       </c>
@@ -1780,7 +1779,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="64" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>64</v>
       </c>
@@ -1794,7 +1793,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="65" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>65</v>
       </c>
@@ -1808,7 +1807,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="66" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>66</v>
       </c>
@@ -1822,7 +1821,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="67" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>67</v>
       </c>
@@ -1836,7 +1835,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="68" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>68</v>
       </c>
@@ -1856,7 +1855,7 @@
         <v>46252</v>
       </c>
     </row>
-    <row r="69" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>69</v>
       </c>
@@ -1870,7 +1869,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="70" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>70</v>
       </c>
@@ -1890,7 +1889,7 @@
         <v>46251</v>
       </c>
     </row>
-    <row r="71" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>71</v>
       </c>
@@ -1904,7 +1903,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="72" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>72</v>
       </c>
@@ -1918,7 +1917,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="73" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>73</v>
       </c>
@@ -1932,7 +1931,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="74" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>74</v>
       </c>
@@ -1946,7 +1945,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="75" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>75</v>
       </c>
@@ -1960,7 +1959,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="76" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>76</v>
       </c>
@@ -1974,7 +1973,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="77" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>77</v>
       </c>
@@ -1988,7 +1987,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="78" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>78</v>
       </c>
@@ -2002,7 +2001,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="79" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>79</v>
       </c>
@@ -2016,7 +2015,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="80" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>80</v>
       </c>
@@ -2030,7 +2029,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="81" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>81</v>
       </c>
@@ -2044,7 +2043,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="82" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>82</v>
       </c>
@@ -2058,7 +2057,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="83" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A83">
         <v>83</v>
       </c>
@@ -2072,7 +2071,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="84" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A84">
         <v>84</v>
       </c>
@@ -2086,7 +2085,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="85" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>85</v>
       </c>
@@ -2100,7 +2099,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="86" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>86</v>
       </c>
@@ -2114,7 +2113,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="87" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>87</v>
       </c>
@@ -2128,7 +2127,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="88" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>88</v>
       </c>
@@ -2142,7 +2141,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="89" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A89">
         <v>89</v>
       </c>
@@ -2156,7 +2155,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="90" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A90">
         <v>90</v>
       </c>
@@ -2170,7 +2169,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="91" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A91">
         <v>91</v>
       </c>
@@ -2184,7 +2183,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="92" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A92">
         <v>92</v>
       </c>
@@ -2198,7 +2197,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="93" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A93">
         <v>93</v>
       </c>
@@ -2212,7 +2211,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="94" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A94">
         <v>94</v>
       </c>
@@ -2226,7 +2225,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="95" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A95">
         <v>95</v>
       </c>
@@ -2240,7 +2239,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="96" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A96">
         <v>96</v>
       </c>
@@ -2254,7 +2253,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="97" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A97">
         <v>97</v>
       </c>
@@ -2268,7 +2267,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="98" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A98">
         <v>98</v>
       </c>
@@ -2288,7 +2287,7 @@
         <v>46224</v>
       </c>
     </row>
-    <row r="99" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A99">
         <v>99</v>
       </c>
@@ -2302,7 +2301,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="100" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>114</v>
       </c>
@@ -2322,7 +2321,7 @@
         <v>46253</v>
       </c>
     </row>
-    <row r="101" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>117</v>
       </c>
@@ -2336,7 +2335,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="102" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>119</v>
       </c>
@@ -2350,7 +2349,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="103" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>121</v>
       </c>
@@ -2364,7 +2363,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="104" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>123</v>
       </c>
@@ -2378,7 +2377,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="105" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>125</v>
       </c>
@@ -2392,7 +2391,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="106" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>127</v>
       </c>
@@ -2406,7 +2405,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="107" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>129</v>
       </c>
@@ -2420,7 +2419,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="108" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>131</v>
       </c>
@@ -2434,7 +2433,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="109" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>133</v>
       </c>
@@ -2448,7 +2447,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="110" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>135</v>
       </c>
@@ -2462,7 +2461,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="111" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>137</v>
       </c>
@@ -2476,7 +2475,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="112" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>139</v>
       </c>
@@ -2490,7 +2489,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="113" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>141</v>
       </c>
@@ -2504,7 +2503,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="114" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>143</v>
       </c>
@@ -2518,7 +2517,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="115" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>145</v>
       </c>
@@ -2532,7 +2531,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="116" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>147</v>
       </c>
@@ -2546,7 +2545,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="117" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>149</v>
       </c>
@@ -2559,8 +2558,14 @@
       <c r="D117" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="118" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+      <c r="E117" t="s">
+        <v>65</v>
+      </c>
+      <c r="F117" s="2">
+        <v>46302</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>151</v>
       </c>
@@ -2574,7 +2579,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="119" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>153</v>
       </c>
@@ -2588,7 +2593,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="120" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>156</v>
       </c>
@@ -2603,18 +2608,20 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F120" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="1">
-      <filters>
-        <filter val="Jovita Alvarado Rafael"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="667d70cb-f49f-4223-87b6-a8a0e4fc3231">
@@ -2623,15 +2630,6 @@
     <TaxCatchAll xmlns="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2842,20 +2840,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{630299A7-E824-4D69-AA5E-3193E7062408}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E73E3A5A-F8DC-40E4-A1F8-9A051C36DEF4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="667d70cb-f49f-4223-87b6-a8a0e4fc3231"/>
     <ds:schemaRef ds:uri="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{630299A7-E824-4D69-AA5E-3193E7062408}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Actualizacion automatica vie 09/10/2026 10:05:56.77
</commit_message>
<xml_diff>
--- a/data/BD Personal.xlsx
+++ b/data/BD Personal.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://apoyoconsultoria0.sharepoint.com/sites/fileserver/Polticas Pblicas/6 Proyectos/2025/2025-070-O IJM - Linea de base/04. Analisis/03. Programacion/06. Dashboard Seguimiento Web/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="41" documentId="11_A10BAE44CD785D61F5141092B1107384533E0B90" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F9295F5B-D81C-4CB2-888E-5597E2499581}"/>
+  <xr:revisionPtr revIDLastSave="44" documentId="11_A10BAE44CD785D61F5141092B1107384533E0B90" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6D82B88C-EE5F-4E6F-B307-0B1934E41B74}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2613,26 +2613,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="667d70cb-f49f-4223-87b6-a8a0e4fc3231">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101007183A11C1BA9EC45BAE4956AD7AAC49F" ma:contentTypeVersion="13" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="07c8fde6007faf37af3ccef690656753">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="667d70cb-f49f-4223-87b6-a8a0e4fc3231" xmlns:ns3="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a1f83a7a0bc9c2dabcf9590cf8de720c" ns2:_="" ns3:_="">
     <xsd:import namespace="667d70cb-f49f-4223-87b6-a8a0e4fc3231"/>
@@ -2839,10 +2819,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="667d70cb-f49f-4223-87b6-a8a0e4fc3231">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{630299A7-E824-4D69-AA5E-3193E7062408}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8ECD6F41-4F89-4BE2-9861-B9B997A6B652}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="667d70cb-f49f-4223-87b6-a8a0e4fc3231"/>
+    <ds:schemaRef ds:uri="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2859,20 +2870,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8ECD6F41-4F89-4BE2-9861-B9B997A6B652}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{630299A7-E824-4D69-AA5E-3193E7062408}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="667d70cb-f49f-4223-87b6-a8a0e4fc3231"/>
-    <ds:schemaRef ds:uri="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizacion automatica mié 14/10/2026  9:37:14.03
</commit_message>
<xml_diff>
--- a/data/BD Personal.xlsx
+++ b/data/BD Personal.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://apoyoconsultoria0.sharepoint.com/sites/fileserver/Polticas Pblicas/6 Proyectos/2025/2025-070-O IJM - Linea de base/04. Analisis/03. Programacion/06. Dashboard Seguimiento Web/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="44" documentId="11_A10BAE44CD785D61F5141092B1107384533E0B90" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6D82B88C-EE5F-4E6F-B307-0B1934E41B74}"/>
+  <xr:revisionPtr revIDLastSave="67" documentId="11_A10BAE44CD785D61F5141092B1107384533E0B90" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FAA49753-3104-4424-B062-D54F48AEA047}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Exported" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Exported!$A$1:$F$120</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Exported!$A$1:$F$124</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="412" uniqueCount="165">
   <si>
     <t>CODPER</t>
   </si>
@@ -507,6 +507,30 @@
   </si>
   <si>
     <t>C0</t>
+  </si>
+  <si>
+    <t>C1</t>
+  </si>
+  <si>
+    <t>C2</t>
+  </si>
+  <si>
+    <t>C3</t>
+  </si>
+  <si>
+    <t>C4</t>
+  </si>
+  <si>
+    <t>Jacqueline Ubillus Torres</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rocío Flores Manrique                                                          </t>
+  </si>
+  <si>
+    <t>C5</t>
+  </si>
+  <si>
+    <t>Evelin Yaranga Villantoy</t>
   </si>
 </sst>
 </file>
@@ -863,7 +887,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F120"/>
+  <dimension ref="A1:F125"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.109375" bestFit="1" customWidth="1"/>
@@ -2607,12 +2631,102 @@
         <v>39</v>
       </c>
     </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A121" t="s">
+        <v>157</v>
+      </c>
+      <c r="B121" t="s">
+        <v>161</v>
+      </c>
+      <c r="C121" t="s">
+        <v>10</v>
+      </c>
+      <c r="D121" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A122" t="s">
+        <v>158</v>
+      </c>
+      <c r="B122" t="s">
+        <v>162</v>
+      </c>
+      <c r="C122" t="s">
+        <v>10</v>
+      </c>
+      <c r="D122" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A123" t="s">
+        <v>159</v>
+      </c>
+      <c r="B123" t="s">
+        <v>106</v>
+      </c>
+      <c r="C123" t="s">
+        <v>10</v>
+      </c>
+      <c r="D123" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A124" t="s">
+        <v>160</v>
+      </c>
+      <c r="B124" t="s">
+        <v>22</v>
+      </c>
+      <c r="C124" t="s">
+        <v>10</v>
+      </c>
+      <c r="D124" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A125" t="s">
+        <v>163</v>
+      </c>
+      <c r="B125" t="s">
+        <v>164</v>
+      </c>
+      <c r="C125" t="s">
+        <v>10</v>
+      </c>
+      <c r="D125" t="s">
+        <v>65</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="667d70cb-f49f-4223-87b6-a8a0e4fc3231">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101007183A11C1BA9EC45BAE4956AD7AAC49F" ma:contentTypeVersion="13" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="07c8fde6007faf37af3ccef690656753">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="667d70cb-f49f-4223-87b6-a8a0e4fc3231" xmlns:ns3="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a1f83a7a0bc9c2dabcf9590cf8de720c" ns2:_="" ns3:_="">
     <xsd:import namespace="667d70cb-f49f-4223-87b6-a8a0e4fc3231"/>
@@ -2819,27 +2933,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="667d70cb-f49f-4223-87b6-a8a0e4fc3231">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{630299A7-E824-4D69-AA5E-3193E7062408}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E73E3A5A-F8DC-40E4-A1F8-9A051C36DEF4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="667d70cb-f49f-4223-87b6-a8a0e4fc3231"/>
+    <ds:schemaRef ds:uri="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8ECD6F41-4F89-4BE2-9861-B9B997A6B652}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2856,23 +2969,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E73E3A5A-F8DC-40E4-A1F8-9A051C36DEF4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="667d70cb-f49f-4223-87b6-a8a0e4fc3231"/>
-    <ds:schemaRef ds:uri="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{630299A7-E824-4D69-AA5E-3193E7062408}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizacion automatica mar 20/10/2026  9:47:26.05
</commit_message>
<xml_diff>
--- a/data/BD Personal.xlsx
+++ b/data/BD Personal.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://apoyoconsultoria0.sharepoint.com/sites/fileserver/Polticas Pblicas/6 Proyectos/2025/2025-070-O IJM - Linea de base/04. Analisis/03. Programacion/06. Dashboard Seguimiento Web/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="67" documentId="11_A10BAE44CD785D61F5141092B1107384533E0B90" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FAA49753-3104-4424-B062-D54F48AEA047}"/>
+  <xr:revisionPtr revIDLastSave="74" documentId="11_A10BAE44CD785D61F5141092B1107384533E0B90" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6AB3613F-2902-4A1F-B320-DC1CF6E8DED3}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Exported" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Exported!$A$1:$F$124</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Exported!$A$1:$F$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="412" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="416" uniqueCount="167">
   <si>
     <t>CODPER</t>
   </si>
@@ -531,6 +531,12 @@
   </si>
   <si>
     <t>Evelin Yaranga Villantoy</t>
+  </si>
+  <si>
+    <t>C6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LUZ MARIA AYALA COBEÑA                                                          </t>
   </si>
 </sst>
 </file>
@@ -887,7 +893,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F125"/>
+  <dimension ref="A1:F126"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.109375" bestFit="1" customWidth="1"/>
@@ -2701,21 +2707,27 @@
         <v>65</v>
       </c>
     </row>
+    <row r="126" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A126" t="s">
+        <v>165</v>
+      </c>
+      <c r="B126" t="s">
+        <v>166</v>
+      </c>
+      <c r="C126" t="s">
+        <v>10</v>
+      </c>
+      <c r="D126" t="s">
+        <v>18</v>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:F1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="667d70cb-f49f-4223-87b6-a8a0e4fc3231">
@@ -2724,6 +2736,15 @@
     <TaxCatchAll xmlns="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2934,20 +2955,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{630299A7-E824-4D69-AA5E-3193E7062408}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E73E3A5A-F8DC-40E4-A1F8-9A051C36DEF4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="667d70cb-f49f-4223-87b6-a8a0e4fc3231"/>
     <ds:schemaRef ds:uri="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{630299A7-E824-4D69-AA5E-3193E7062408}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Actualizacion automatica mar 20/10/2026  9:51:23.90
</commit_message>
<xml_diff>
--- a/data/BD Personal.xlsx
+++ b/data/BD Personal.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://apoyoconsultoria0.sharepoint.com/sites/fileserver/Polticas Pblicas/6 Proyectos/2025/2025-070-O IJM - Linea de base/04. Analisis/03. Programacion/06. Dashboard Seguimiento Web/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="74" documentId="11_A10BAE44CD785D61F5141092B1107384533E0B90" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6AB3613F-2902-4A1F-B320-DC1CF6E8DED3}"/>
+  <xr:revisionPtr revIDLastSave="75" documentId="11_A10BAE44CD785D61F5141092B1107384533E0B90" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F9047CBF-AAFD-4490-B6DE-D6FB3401C455}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -536,7 +536,7 @@
     <t>C6</t>
   </si>
   <si>
-    <t xml:space="preserve">LUZ MARIA AYALA COBEÑA                                                          </t>
+    <t>LUZ MARIA AYALA COBEÑA</t>
   </si>
 </sst>
 </file>
@@ -2728,6 +2728,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="667d70cb-f49f-4223-87b6-a8a0e4fc3231">
@@ -2736,15 +2745,6 @@
     <TaxCatchAll xmlns="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2955,20 +2955,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{630299A7-E824-4D69-AA5E-3193E7062408}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E73E3A5A-F8DC-40E4-A1F8-9A051C36DEF4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="667d70cb-f49f-4223-87b6-a8a0e4fc3231"/>
     <ds:schemaRef ds:uri="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{630299A7-E824-4D69-AA5E-3193E7062408}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>